<commit_message>
feat(audio): 数据驱动音频系统(Luban Audio 表 + AudioConfigMgr)
骑在 TEngine 内置 AudioModule 之上加数据驱动配置层,不重造通道池/播放。
- Luban: 新增 audio.TbAudio(9 字段)+ EAudioType/EAudioGroup/EAudioFade 枚举 + 4 行样板;Global 表加 DefaultCooldown(id=6)
- AudioConfigMgr: 按 id 播放,Type→AudioType 路由、Volume/Loop 透传、Cooldown 防连点门(专属覆盖全局)、AudioGroup⊆Type 加载期校验、FadeInOut best-effort(淡入协程以 AudioData 引用作播放令牌防抢占误写)
- GlobalConfigMgr: 补 AudioDefaultCooldown 便捷属性
- EditMode 测试 17 项(纯逻辑 + 直读 audio_tbaudio.bytes)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/__enums__.xlsx
+++ b/Configs/GameConfig/Datas/__enums__.xlsx
@@ -1092,7 +1092,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:L43"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" style="4" min="2" max="2"/>
@@ -1684,96 +1684,336 @@
       <c r="K27" s="0" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="0" t="inlineStr">
         <is>
           <t>avatar.EAvatarType</t>
         </is>
       </c>
-      <c r="C28" t="b">
+      <c r="C28" s="0" t="b">
         <v>0</v>
       </c>
-      <c r="D28" t="b">
+      <c r="D28" s="0" t="b">
         <v>1</v>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="G28" s="0" t="inlineStr">
         <is>
           <t>头像类型(1头像2头像框)</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
+      <c r="H28" s="0" t="inlineStr">
         <is>
           <t>AVATAR</t>
         </is>
       </c>
-      <c r="J28" t="n">
+      <c r="J28" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="K28" t="inlineStr">
+      <c r="K28" s="0" t="inlineStr">
         <is>
           <t>头像</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="H29" t="inlineStr">
+      <c r="H29" s="0" t="inlineStr">
         <is>
           <t>FRAME</t>
         </is>
       </c>
-      <c r="J29" t="n">
+      <c r="J29" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="K29" t="inlineStr">
+      <c r="K29" s="0" t="inlineStr">
         <is>
           <t>头像框</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="0" t="inlineStr">
         <is>
           <t>avatar.EUnlockCond</t>
         </is>
       </c>
-      <c r="C30" t="b">
+      <c r="C30" s="0" t="b">
         <v>0</v>
       </c>
-      <c r="D30" t="b">
+      <c r="D30" s="0" t="b">
         <v>1</v>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="G30" s="0" t="inlineStr">
         <is>
           <t>解锁条件(1等级2活动发放)</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
+      <c r="H30" s="0" t="inlineStr">
         <is>
           <t>LEVEL</t>
         </is>
       </c>
-      <c r="J30" t="n">
+      <c r="J30" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="K30" t="inlineStr">
+      <c r="K30" s="0" t="inlineStr">
         <is>
           <t>等级解锁</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="H31" t="inlineStr">
+      <c r="H31" s="0" t="inlineStr">
         <is>
           <t>EVENT</t>
         </is>
       </c>
-      <c r="J31" t="n">
+      <c r="J31" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="K31" t="inlineStr">
+      <c r="K31" s="0" t="inlineStr">
         <is>
           <t>活动发放</t>
         </is>
       </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>audio.EAudioType</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="b">
+        <v>0</v>
+      </c>
+      <c r="D32" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="G32" s="0" t="inlineStr">
+        <is>
+          <t>音频粗分类(决定通道池/播放策略)</t>
+        </is>
+      </c>
+      <c r="H32" s="0" t="inlineStr">
+        <is>
+          <t>BGM</t>
+        </is>
+      </c>
+      <c r="I32" s="0" t="inlineStr">
+        <is>
+          <t>背景音乐</t>
+        </is>
+      </c>
+      <c r="J32" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" s="0" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="H33" s="0" t="inlineStr">
+        <is>
+          <t>GlobalUI</t>
+        </is>
+      </c>
+      <c r="I33" s="0" t="inlineStr">
+        <is>
+          <t>全局UI音效</t>
+        </is>
+      </c>
+      <c r="J33" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="K33" s="0" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="H34" s="0" t="inlineStr">
+        <is>
+          <t>InGame</t>
+        </is>
+      </c>
+      <c r="I34" s="0" t="inlineStr">
+        <is>
+          <t>局内玩法音效</t>
+        </is>
+      </c>
+      <c r="J34" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="K34" s="0" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>audio.EAudioGroup</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="b">
+        <v>0</v>
+      </c>
+      <c r="D35" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="G35" s="0" t="inlineStr">
+        <is>
+          <t>音频混音分组(Type的子类型)</t>
+        </is>
+      </c>
+      <c r="H35" s="0" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="I35" s="0" t="inlineStr">
+        <is>
+          <t>全局</t>
+        </is>
+      </c>
+      <c r="J35" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" s="0" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="H36" s="0" t="inlineStr">
+        <is>
+          <t>BGM</t>
+        </is>
+      </c>
+      <c r="I36" s="0" t="inlineStr">
+        <is>
+          <t>背景音乐</t>
+        </is>
+      </c>
+      <c r="J36" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="K36" s="0" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="H37" s="0" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="I37" s="0" t="inlineStr">
+        <is>
+          <t>界面</t>
+        </is>
+      </c>
+      <c r="J37" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="K37" s="0" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="H38" s="0" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+      <c r="I38" s="0" t="inlineStr">
+        <is>
+          <t>战斗</t>
+        </is>
+      </c>
+      <c r="J38" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="K38" s="0" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="H39" s="0" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="I39" s="0" t="inlineStr">
+        <is>
+          <t>语音</t>
+        </is>
+      </c>
+      <c r="J39" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="K39" s="0" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>audio.EAudioFade</t>
+        </is>
+      </c>
+      <c r="C40" t="b">
+        <v>0</v>
+      </c>
+      <c r="D40" t="b">
+        <v>1</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>淡入淡出模式</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="J40" t="n">
+        <v>0</v>
+      </c>
+      <c r="K40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>In</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>仅淡入</t>
+        </is>
+      </c>
+      <c r="J41" t="n">
+        <v>1</v>
+      </c>
+      <c r="K41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Out</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>仅淡出</t>
+        </is>
+      </c>
+      <c r="J42" t="n">
+        <v>2</v>
+      </c>
+      <c r="K42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>双向</t>
+        </is>
+      </c>
+      <c r="J43" t="n">
+        <v>3</v>
+      </c>
+      <c r="K43" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>